<commit_message>
Export ISA validation results to JSON
Modified alarm_analytics.py to return structured validation results from the test case validation method and persist them to a JSON file. Added configuration entry for the new output file. This enables downstream processes to programmatically access test validation outcomes (chattering, stale, cluster detection).
</commit_message>
<xml_diff>
--- a/scripts/analytics-pipeline/output/data_dictionary.xlsx
+++ b/scripts/analytics-pipeline/output/data_dictionary.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="86">
   <si>
     <t>Column</t>
   </si>
@@ -141,6 +141,9 @@
     <t>Nulls retained; flagged as missing</t>
   </si>
   <si>
+    <t>Nullable (NULL for real-world data)</t>
+  </si>
+  <si>
     <t>pass | missing | outlier</t>
   </si>
   <si>
@@ -186,6 +189,12 @@
     <t>priority</t>
   </si>
   <si>
+    <t>ack_time</t>
+  </si>
+  <si>
+    <t>clear_time</t>
+  </si>
+  <si>
     <t>duration_min</t>
   </si>
   <si>
@@ -219,7 +228,13 @@
     <t>Event-driven</t>
   </si>
   <si>
-    <t>Mostly null in source</t>
+    <t>Nullable (NULL if not acknowledged)</t>
+  </si>
+  <si>
+    <t>Nullable (NULL if still active)</t>
+  </si>
+  <si>
+    <t>Nullable</t>
   </si>
   <si>
     <t>HI | LO</t>
@@ -255,10 +270,10 @@
     <t>5-min</t>
   </si>
   <si>
-    <t>1.00 to 105299.00</t>
-  </si>
-  <si>
-    <t>750.00 to 45400.00</t>
+    <t>1.00 to 105399.00</t>
+  </si>
+  <si>
+    <t>750.00 to 156000.00</t>
   </si>
 </sst>
 </file>
@@ -681,7 +696,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -752,10 +767,10 @@
         <v>40</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -778,10 +793,10 @@
         <v>40</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -804,10 +819,10 @@
         <v>40</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -830,10 +845,10 @@
         <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -856,10 +871,10 @@
         <v>40</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -882,10 +897,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -908,10 +923,10 @@
         <v>40</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -934,10 +949,10 @@
         <v>40</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -957,10 +972,10 @@
         <v>38</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>25</v>
@@ -986,7 +1001,7 @@
         <v>39</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>25</v>
@@ -999,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -1055,7 +1070,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1069,10 +1084,10 @@
         <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>39</v>
@@ -1093,10 +1108,10 @@
         <v>25</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>39</v>
@@ -1108,19 +1123,19 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>39</v>
@@ -1132,19 +1147,19 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>39</v>
@@ -1156,25 +1171,25 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>25</v>
@@ -1182,7 +1197,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>21</v>
@@ -1191,63 +1206,63 @@
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2" t="s">
@@ -1256,31 +1271,31 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>63</v>
@@ -1289,13 +1304,13 @@
         <v>25</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
@@ -1304,27 +1319,75 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1391,7 +1454,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1405,10 +1468,10 @@
         <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>39</v>
@@ -1420,28 +1483,28 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>40</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1449,7 +1512,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
@@ -1464,7 +1527,7 @@
         <v>39</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>25</v>

</xml_diff>